<commit_message>
feat: botones descarga, roles nuevos, mapa leaflet, latitud/longitud PDV y paquete base de datos
</commit_message>
<xml_diff>
--- a/Backend/visitapp_backend/src/assets/plantilla_pdv.xlsx
+++ b/Backend/visitapp_backend/src/assets/plantilla_pdv.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectosFlutter\visitasapp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectosFlutter\Backoffice_work\Backend\visitapp_backend\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{297167D0-FED3-4F19-B992-B958678EC6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{64E8FBD6-E05B-4D82-8147-F98D97353B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,16 +18,17 @@
     <sheet name="Resultado esperado en BD" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="85">
   <si>
     <t>CARGA MASIVA — PUNTOS DE VENTA</t>
   </si>
   <si>
-    <t>Instrucciones: Complete una fila por cada Punto de Venta. Los campos marcados con * son obligatorios. La MAC debe tener formato XX:XX:XX:XX:XX:XX. No modifique los encabezados.</t>
+    <t>Instrucciones: Complete una fila por cada Punto de Venta. Los campos marcados con * son obligatorios. La MAC debe tener formato XX:XX:XX:XX:XX:XX. Latitud y Longitud son opcionales. No modifique los encabezados.</t>
   </si>
   <si>
     <t>DEPARTAMENTO *</t>
@@ -54,6 +55,12 @@
     <t>DIRECCIÓN</t>
   </si>
   <si>
+    <t>LATITUD</t>
+  </si>
+  <si>
+    <t>LONGITUD</t>
+  </si>
+  <si>
     <t>Cundinamarca</t>
   </si>
   <si>
@@ -247,6 +254,30 @@
   </si>
   <si>
     <t>Punto de Venta</t>
+  </si>
+  <si>
+    <t>ARAUCA</t>
+  </si>
+  <si>
+    <t>CASANARE</t>
+  </si>
+  <si>
+    <t>GUAVIARE</t>
+  </si>
+  <si>
+    <t>GUAINIA</t>
+  </si>
+  <si>
+    <t>SAN ANDRES</t>
+  </si>
+  <si>
+    <t>Zona 1</t>
+  </si>
+  <si>
+    <t>Oficina principal</t>
+  </si>
+  <si>
+    <t>PDV Principal</t>
   </si>
 </sst>
 </file>
@@ -402,12 +433,12 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -717,7 +748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -726,10 +757,11 @@
     <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="35" customWidth="1"/>
+    <col min="9" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:10" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="10"/>
@@ -739,9 +771,11 @@
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
-    </row>
-    <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="10"/>
@@ -751,8 +785,10 @@
       <c r="F2" s="10"/>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
-    </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+    </row>
+    <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -777,138 +813,174 @@
       <c r="H3" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>77</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="2">
+        <v>4.6486000000000001</v>
+      </c>
+      <c r="J4" s="2">
+        <v>-74.063299999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>19</v>
+      <c r="E5" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="I5" s="3">
+        <v>4.6486000000000001</v>
+      </c>
+      <c r="J5" s="3">
+        <v>-74.063299999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="I6" s="2">
+        <v>4.6486000000000001</v>
+      </c>
+      <c r="J6" s="2">
+        <v>-74.063299999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="3" t="s">
         <v>34</v>
       </c>
+      <c r="E7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="G7" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="I7" s="3">
+        <v>4.6486000000000001</v>
+      </c>
+      <c r="J7" s="3">
+        <v>-74.063299999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="I8" s="2">
+        <v>4.6486000000000001</v>
+      </c>
+      <c r="J8" s="2">
+        <v>-74.063299999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -917,8 +989,10 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -927,8 +1001,10 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -937,8 +1013,10 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -947,8 +1025,10 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -957,8 +1037,10 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -967,8 +1049,10 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -977,8 +1061,10 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -987,8 +1073,10 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -997,8 +1085,10 @@
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1007,8 +1097,10 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1017,8 +1109,10 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1027,8 +1121,10 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1037,8 +1133,10 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1047,8 +1145,10 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1057,8 +1157,10 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1067,8 +1169,10 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1077,8 +1181,10 @@
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1087,8 +1193,10 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1097,8 +1205,10 @@
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1107,8 +1217,10 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1117,8 +1229,10 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1127,8 +1241,10 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1137,8 +1253,10 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1147,8 +1265,10 @@
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1157,8 +1277,10 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1167,8 +1289,10 @@
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1177,8 +1301,10 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1187,8 +1313,10 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1197,8 +1325,10 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1207,8 +1337,10 @@
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1217,8 +1349,10 @@
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1227,8 +1361,10 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1237,8 +1373,10 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -1247,8 +1385,10 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1257,8 +1397,10 @@
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1267,8 +1409,10 @@
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1277,8 +1421,10 @@
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1287,8 +1433,10 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1297,8 +1445,10 @@
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -1307,8 +1457,10 @@
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1317,8 +1469,10 @@
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -1327,8 +1481,10 @@
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1337,8 +1493,10 @@
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -1347,8 +1505,10 @@
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1357,8 +1517,10 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -1367,8 +1529,10 @@
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1377,8 +1541,10 @@
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
       <c r="H55" s="3"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -1387,8 +1553,10 @@
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -1397,8 +1565,10 @@
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -1407,8 +1577,10 @@
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -1417,8 +1589,10 @@
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -1427,8 +1601,10 @@
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -1437,8 +1613,10 @@
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I61" s="3"/>
+      <c r="J61" s="3"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -1447,8 +1625,10 @@
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I62" s="2"/>
+      <c r="J62" s="2"/>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -1457,8 +1637,10 @@
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -1467,8 +1649,10 @@
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I64" s="2"/>
+      <c r="J64" s="2"/>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -1477,8 +1661,10 @@
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I65" s="3"/>
+      <c r="J65" s="3"/>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -1487,8 +1673,10 @@
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -1497,8 +1685,10 @@
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
       <c r="H67" s="3"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -1507,8 +1697,10 @@
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I68" s="2"/>
+      <c r="J68" s="2"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -1517,8 +1709,10 @@
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
       <c r="H69" s="3"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -1527,8 +1721,10 @@
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I70" s="2"/>
+      <c r="J70" s="2"/>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -1537,8 +1733,10 @@
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
       <c r="H71" s="3"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I71" s="3"/>
+      <c r="J71" s="3"/>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -1547,8 +1745,10 @@
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I72" s="2"/>
+      <c r="J72" s="2"/>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -1557,8 +1757,10 @@
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
       <c r="H73" s="3"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -1567,8 +1769,10 @@
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I74" s="2"/>
+      <c r="J74" s="2"/>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -1577,8 +1781,10 @@
       <c r="F75" s="3"/>
       <c r="G75" s="3"/>
       <c r="H75" s="3"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -1587,8 +1793,10 @@
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I76" s="2"/>
+      <c r="J76" s="2"/>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -1597,8 +1805,10 @@
       <c r="F77" s="3"/>
       <c r="G77" s="3"/>
       <c r="H77" s="3"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I77" s="3"/>
+      <c r="J77" s="3"/>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -1607,8 +1817,10 @@
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I78" s="2"/>
+      <c r="J78" s="2"/>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -1617,8 +1829,10 @@
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -1627,8 +1841,10 @@
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I80" s="2"/>
+      <c r="J80" s="2"/>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -1637,8 +1853,10 @@
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
       <c r="H81" s="3"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -1647,8 +1865,10 @@
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I82" s="2"/>
+      <c r="J82" s="2"/>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -1657,8 +1877,10 @@
       <c r="F83" s="3"/>
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I83" s="3"/>
+      <c r="J83" s="3"/>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -1667,8 +1889,10 @@
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I84" s="2"/>
+      <c r="J84" s="2"/>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -1677,8 +1901,10 @@
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I85" s="3"/>
+      <c r="J85" s="3"/>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -1687,8 +1913,10 @@
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I86" s="2"/>
+      <c r="J86" s="2"/>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -1697,8 +1925,10 @@
       <c r="F87" s="3"/>
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I87" s="3"/>
+      <c r="J87" s="3"/>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -1707,8 +1937,10 @@
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I88" s="2"/>
+      <c r="J88" s="2"/>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -1717,8 +1949,10 @@
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I89" s="3"/>
+      <c r="J89" s="3"/>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -1727,8 +1961,10 @@
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I90" s="2"/>
+      <c r="J90" s="2"/>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -1737,8 +1973,10 @@
       <c r="F91" s="3"/>
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I91" s="3"/>
+      <c r="J91" s="3"/>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -1747,8 +1985,10 @@
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I92" s="2"/>
+      <c r="J92" s="2"/>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -1757,8 +1997,10 @@
       <c r="F93" s="3"/>
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I93" s="3"/>
+      <c r="J93" s="3"/>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -1767,8 +2009,10 @@
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I94" s="2"/>
+      <c r="J94" s="2"/>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -1777,8 +2021,10 @@
       <c r="F95" s="3"/>
       <c r="G95" s="3"/>
       <c r="H95" s="3"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I95" s="3"/>
+      <c r="J95" s="3"/>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -1787,8 +2033,10 @@
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I96" s="2"/>
+      <c r="J96" s="2"/>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -1797,8 +2045,10 @@
       <c r="F97" s="3"/>
       <c r="G97" s="3"/>
       <c r="H97" s="3"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I97" s="3"/>
+      <c r="J97" s="3"/>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -1807,8 +2057,10 @@
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I98" s="2"/>
+      <c r="J98" s="2"/>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -1817,8 +2069,10 @@
       <c r="F99" s="3"/>
       <c r="G99" s="3"/>
       <c r="H99" s="3"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I99" s="3"/>
+      <c r="J99" s="3"/>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -1827,8 +2081,10 @@
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I100" s="2"/>
+      <c r="J100" s="2"/>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -1837,8 +2093,10 @@
       <c r="F101" s="3"/>
       <c r="G101" s="3"/>
       <c r="H101" s="3"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I101" s="3"/>
+      <c r="J101" s="3"/>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -1847,8 +2105,10 @@
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I102" s="2"/>
+      <c r="J102" s="2"/>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -1860,8 +2120,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1878,16 +2138,16 @@
   <sheetData>
     <row r="1" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B1" s="10"/>
     </row>
     <row r="2" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1896,10 +2156,10 @@
     </row>
     <row r="4" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1907,7 +2167,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1915,7 +2175,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1923,7 +2183,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1931,7 +2191,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1939,7 +2199,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1947,7 +2207,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1955,7 +2215,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1963,7 +2223,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1972,22 +2232,22 @@
     </row>
     <row r="14" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1996,34 +2256,34 @@
     </row>
     <row r="18" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2047,7 +2307,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -2057,122 +2317,122 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>